<commit_message>
Update route UI and deck data
</commit_message>
<xml_diff>
--- a/Data/carddesign.xlsx
+++ b/Data/carddesign.xlsx
@@ -8,13 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\TapMiniGame\CardLoot\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{688B39BC-A69D-41FB-83F2-C610F93B705E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D2FDD5E-9FF7-46ED-B066-F7D45F6B5610}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10988" yWindow="0" windowWidth="8295" windowHeight="11363" xr2:uid="{D71E6DA9-D267-45CD-9DB8-FB5FB51F7F48}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{D71E6DA9-D267-45CD-9DB8-FB5FB51F7F48}"/>
   </bookViews>
   <sheets>
     <sheet name="全卡表" sheetId="2" r:id="rId1"/>
-    <sheet name="轮1卡组" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="48">
   <si>
     <t>效果名</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -107,10 +106,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>埋伏</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>复制</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -123,26 +118,10 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>汲取</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>洪水</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>污染</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>威吓</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>怂恿</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>废土</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -175,10 +154,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>盾牌</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>是否解锁</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -207,19 +182,50 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>普通</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>扒手</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>流浪汉</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>迷失者</t>
+    <t>一分</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>三分</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>牌名</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>二分</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>贷款</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>陷阱</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>回收</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>勾引</t>
+  </si>
+  <si>
+    <t>魅魔</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>掀桌</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>被动：对手队列中每有1个炸弹，自身+3分</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>泄密</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -613,466 +619,524 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6EBCBEC8-5D21-4A68-9874-E023DEBF469A}">
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="2" width="16.3984375" customWidth="1"/>
-    <col min="3" max="3" width="10.46484375" customWidth="1"/>
-    <col min="5" max="5" width="11.86328125" customWidth="1"/>
-    <col min="6" max="6" width="43.53125" customWidth="1"/>
+    <col min="1" max="3" width="16.3984375" customWidth="1"/>
+    <col min="4" max="4" width="10.46484375" customWidth="1"/>
+    <col min="6" max="6" width="11.86328125" customWidth="1"/>
+    <col min="7" max="7" width="43.53125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="B1" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1" t="s">
         <v>13</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>7</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>0</v>
       </c>
-      <c r="F1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A2" s="1">
         <v>1</v>
       </c>
-      <c r="B2" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="C2">
+      <c r="B2" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C2" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="D2">
         <v>2</v>
       </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="E2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A3" s="1">
         <v>2</v>
       </c>
-      <c r="B3" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="C3">
+      <c r="B3" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C3" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="D3">
         <v>4</v>
       </c>
-      <c r="D3">
+      <c r="E3">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A4" s="1">
         <v>3</v>
       </c>
-      <c r="B4" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="C4">
+      <c r="B4" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C4" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="D4">
         <v>6</v>
       </c>
-      <c r="D4">
+      <c r="E4">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A5" s="1">
         <v>4</v>
       </c>
-      <c r="B5" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="C5">
+      <c r="B5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C5" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="D5">
         <v>5</v>
       </c>
-      <c r="D5">
+      <c r="E5">
         <v>-1</v>
       </c>
-      <c r="E5" t="s">
-        <v>17</v>
-      </c>
       <c r="F5" t="s">
+        <v>41</v>
+      </c>
+      <c r="G5" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A6" s="1">
         <v>5</v>
       </c>
-      <c r="B6" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="C6">
+      <c r="B6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="D6">
         <v>5</v>
       </c>
-      <c r="D6">
-        <v>1</v>
-      </c>
-      <c r="E6" t="s">
-        <v>18</v>
+      <c r="E6">
+        <v>1</v>
       </c>
       <c r="F6" t="s">
+        <v>17</v>
+      </c>
+      <c r="G6" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A7" s="1">
         <v>6</v>
       </c>
-      <c r="B7" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="C7">
-        <v>5</v>
+      <c r="B7" t="s">
+        <v>25</v>
+      </c>
+      <c r="C7" s="1" t="b">
+        <v>1</v>
       </c>
       <c r="D7">
         <v>5</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7">
+        <v>5</v>
+      </c>
+      <c r="F7" t="s">
+        <v>25</v>
+      </c>
+      <c r="G7" t="s">
         <v>30</v>
       </c>
-      <c r="F7" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.4">
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A8" s="1">
         <v>7</v>
       </c>
-      <c r="B8" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="C8">
+      <c r="B8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="D8">
         <v>5</v>
       </c>
-      <c r="D8">
-        <v>1</v>
-      </c>
-      <c r="E8" t="s">
-        <v>19</v>
+      <c r="E8">
+        <v>1</v>
       </c>
       <c r="F8" t="s">
+        <v>18</v>
+      </c>
+      <c r="G8" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A9" s="1">
         <v>8</v>
       </c>
-      <c r="B9" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="C9">
+      <c r="B9" t="s">
+        <v>19</v>
+      </c>
+      <c r="C9" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="D9">
         <v>4</v>
       </c>
-      <c r="D9">
-        <v>1</v>
-      </c>
-      <c r="E9" t="s">
-        <v>20</v>
+      <c r="E9">
+        <v>1</v>
       </c>
       <c r="F9" t="s">
+        <v>19</v>
+      </c>
+      <c r="G9" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A10" s="1">
         <v>9</v>
       </c>
-      <c r="B10" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="C10">
+      <c r="B10" t="s">
+        <v>23</v>
+      </c>
+      <c r="C10" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="D10">
         <v>9</v>
       </c>
-      <c r="D10">
+      <c r="E10">
         <v>2</v>
       </c>
-      <c r="E10" t="s">
-        <v>28</v>
-      </c>
       <c r="F10" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.4">
+        <v>23</v>
+      </c>
+      <c r="G10" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A11" s="1">
         <v>10</v>
       </c>
-      <c r="B11" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="C11">
+      <c r="B11" t="s">
+        <v>42</v>
+      </c>
+      <c r="C11" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="D11">
         <v>4</v>
       </c>
-      <c r="D11">
-        <v>1</v>
-      </c>
-      <c r="E11" t="s">
-        <v>34</v>
+      <c r="E11">
+        <v>1</v>
       </c>
       <c r="F11" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.4">
+        <v>42</v>
+      </c>
+      <c r="G11" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A12" s="1">
         <v>11</v>
       </c>
-      <c r="B12" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="C12">
+      <c r="B12" t="s">
+        <v>26</v>
+      </c>
+      <c r="C12" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="D12">
         <v>5</v>
       </c>
-      <c r="D12">
+      <c r="E12">
         <v>0</v>
       </c>
-      <c r="E12" t="s">
-        <v>31</v>
-      </c>
       <c r="F12" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.4">
+        <v>26</v>
+      </c>
+      <c r="G12" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A13" s="1">
         <v>12</v>
       </c>
-      <c r="B13" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="C13">
+      <c r="B13" t="s">
+        <v>2</v>
+      </c>
+      <c r="C13" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="D13">
         <v>5</v>
       </c>
-      <c r="D13">
+      <c r="E13">
         <v>0</v>
       </c>
-      <c r="E13" t="s">
+      <c r="F13" t="s">
         <v>2</v>
       </c>
-      <c r="F13" t="s">
+      <c r="G13" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A14" s="1">
         <v>13</v>
       </c>
-      <c r="B14" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="C14">
+      <c r="B14" t="s">
+        <v>3</v>
+      </c>
+      <c r="C14" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="D14">
         <v>4</v>
       </c>
-      <c r="D14">
-        <v>1</v>
-      </c>
-      <c r="E14" t="s">
+      <c r="E14">
+        <v>1</v>
+      </c>
+      <c r="F14" t="s">
         <v>3</v>
       </c>
-      <c r="F14" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G14" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A15" s="1">
         <v>14</v>
       </c>
-      <c r="B15" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="C15">
+      <c r="B15" t="s">
+        <v>6</v>
+      </c>
+      <c r="C15" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="D15">
         <v>3</v>
       </c>
-      <c r="D15">
+      <c r="E15">
         <v>0</v>
       </c>
-      <c r="E15" t="s">
+      <c r="F15" t="s">
         <v>6</v>
       </c>
-      <c r="F15" t="s">
+      <c r="G15" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A16" s="1">
         <v>15</v>
       </c>
-      <c r="B16" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="C16">
+      <c r="B16" t="s">
+        <v>44</v>
+      </c>
+      <c r="C16" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="D16">
         <v>5</v>
       </c>
-      <c r="D16">
+      <c r="E16">
         <v>0</v>
       </c>
-      <c r="E16" t="s">
-        <v>21</v>
-      </c>
       <c r="F16" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.4">
+        <v>44</v>
+      </c>
+      <c r="G16" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A17" s="1">
         <v>16</v>
       </c>
-      <c r="B17" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="C17">
+      <c r="B17" t="s">
+        <v>45</v>
+      </c>
+      <c r="C17" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="D17">
         <v>6</v>
       </c>
-      <c r="D17">
+      <c r="E17">
         <v>0</v>
       </c>
-      <c r="E17" t="s">
-        <v>22</v>
-      </c>
       <c r="F17" t="s">
+        <v>45</v>
+      </c>
+      <c r="G17" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A18" s="1">
         <v>17</v>
       </c>
-      <c r="B18" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="C18">
+      <c r="B18" t="s">
+        <v>20</v>
+      </c>
+      <c r="C18" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="D18">
         <v>4</v>
       </c>
-      <c r="D18">
-        <v>1</v>
-      </c>
-      <c r="E18" t="s">
-        <v>23</v>
+      <c r="E18">
+        <v>1</v>
       </c>
       <c r="F18" t="s">
+        <v>20</v>
+      </c>
+      <c r="G18" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A19" s="1">
         <v>18</v>
       </c>
-      <c r="B19" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="C19">
-        <v>4</v>
+      <c r="B19" t="s">
+        <v>40</v>
+      </c>
+      <c r="C19" s="1" t="b">
+        <v>1</v>
       </c>
       <c r="D19">
         <v>4</v>
       </c>
-      <c r="E19" t="s">
-        <v>24</v>
+      <c r="E19">
+        <v>4</v>
       </c>
       <c r="F19" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G19" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A20" s="1">
         <v>19</v>
       </c>
-      <c r="B20" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="C20">
+      <c r="B20" t="s">
+        <v>43</v>
+      </c>
+      <c r="C20" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="D20">
         <v>3</v>
       </c>
-      <c r="D20">
-        <v>1</v>
-      </c>
-      <c r="E20" t="s">
-        <v>25</v>
+      <c r="E20">
+        <v>1</v>
       </c>
       <c r="F20" t="s">
+        <v>43</v>
+      </c>
+      <c r="G20" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A21" s="1">
         <v>20</v>
       </c>
-      <c r="B21" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="C21">
+      <c r="B21" t="s">
+        <v>21</v>
+      </c>
+      <c r="C21" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="D21">
         <v>4</v>
       </c>
-      <c r="D21">
-        <v>1</v>
-      </c>
-      <c r="E21" t="s">
-        <v>26</v>
+      <c r="E21">
+        <v>1</v>
       </c>
       <c r="F21" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.4">
+        <v>21</v>
+      </c>
+      <c r="G21" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A22" s="1">
         <v>21</v>
       </c>
-      <c r="B22" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="C22">
+      <c r="B22" t="s">
+        <v>22</v>
+      </c>
+      <c r="C22" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="D22">
         <v>6</v>
       </c>
-      <c r="D22">
+      <c r="E22">
         <v>2</v>
       </c>
-      <c r="E22" t="s">
-        <v>27</v>
-      </c>
       <c r="F22" t="s">
+        <v>22</v>
+      </c>
+      <c r="G22" t="s">
         <v>11</v>
       </c>
     </row>
-  </sheetData>
-  <phoneticPr fontId="1" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2652BD7C-792B-4508-9BA4-1D4F46003412}">
-  <dimension ref="A1:A4"/>
-  <sheetFormatPr defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
-  <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.4">
-      <c r="A1" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.4">
-      <c r="A2" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.4">
-      <c r="A3" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.4">
-      <c r="A4" t="s">
-        <v>44</v>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A23" s="1">
+        <v>22</v>
+      </c>
+      <c r="B23" t="s">
+        <v>47</v>
+      </c>
+      <c r="C23" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="D23">
+        <v>8</v>
+      </c>
+      <c r="E23">
+        <v>0</v>
+      </c>
+      <c r="F23" t="s">
+        <v>47</v>
+      </c>
+      <c r="G23" t="s">
+        <v>46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Polish game UI and update deck data
</commit_message>
<xml_diff>
--- a/Data/carddesign.xlsx
+++ b/Data/carddesign.xlsx
@@ -2,231 +2,168 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\TapMiniGame\CardLoot\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D2FDD5E-9FF7-46ED-B066-F7D45F6B5610}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEBABE09-4AD7-490C-A8B6-121558E0EC59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{D71E6DA9-D267-45CD-9DB8-FB5FB51F7F48}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="全卡表" sheetId="2" r:id="rId1"/>
+    <sheet name="全卡表" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="48">
   <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>牌名</t>
+  </si>
+  <si>
+    <t>是否解锁</t>
+  </si>
+  <si>
+    <t>商店价格</t>
+  </si>
+  <si>
+    <t>基础分</t>
+  </si>
+  <si>
     <t>效果名</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>效果</t>
-    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>一分</t>
+  </si>
+  <si>
+    <t>二分</t>
+  </si>
+  <si>
+    <t>三分</t>
+  </si>
+  <si>
+    <t>陷阱</t>
+  </si>
+  <si>
+    <t>弃置：往对手抽牌堆中放入一枚“临时”炸弹</t>
+  </si>
+  <si>
+    <t>复制</t>
+  </si>
+  <si>
+    <t>主动：复制自己队列中的一张卡，具有临时效果</t>
+  </si>
+  <si>
+    <t>莽夫</t>
+  </si>
+  <si>
+    <t>被动：被抽取时，会立即再抽2张</t>
+  </si>
+  <si>
+    <t>先锋</t>
+  </si>
+  <si>
+    <t>被动：此后抽取的卡获得+1分</t>
+  </si>
+  <si>
+    <t>小鬼</t>
+  </si>
+  <si>
+    <t>被动：如果是最后一张，则+3分</t>
+  </si>
+  <si>
+    <t>圣光</t>
+  </si>
+  <si>
+    <t>主动：使队列中其他卡牌获得+1分</t>
+  </si>
+  <si>
+    <t>回收</t>
+  </si>
+  <si>
+    <t>主动：选择队列中另外一张卡，将其洗回抽牌堆</t>
+  </si>
+  <si>
+    <t>首领</t>
+  </si>
+  <si>
+    <t>被动：队列中每有1个分数低于2的卡牌，则自身+1分</t>
   </si>
   <si>
     <t>偷窃</t>
-    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>主动：选择对手队列中的一个卡，将其放入自身的队列（弃牌后返回对手弃牌堆）</t>
   </si>
   <si>
     <t>虚张</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>主动：选择对手队列中的一个卡，将其放入自身的队列（弃牌后返回对手弃牌堆）</t>
-    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>被动:如果对手的队列数量小于等于3，则自身+2分</t>
+  </si>
+  <si>
+    <t>恐吓</t>
   </si>
   <si>
     <t>主动：随机弃掉对手队列中的一个卡</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>恐吓</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>基础分</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>弃置：往对手抽牌堆中放入一枚“临时”炸弹</t>
-    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>魅魔</t>
+  </si>
+  <si>
+    <t>被动：在队列中时，对手每再抽一张，则自身+1分</t>
+  </si>
+  <si>
+    <t>掀桌</t>
   </si>
   <si>
     <t>主动：双方各随机弃2张牌</t>
-    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>污染</t>
   </si>
   <si>
     <t>主动：往对手弃牌堆中，加入一张“污染”（具有临时效果，-1分）</t>
-    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>贷款</t>
+  </si>
+  <si>
+    <t>被动：在队列中时，对手每再抽一张，则自身-1分</t>
+  </si>
+  <si>
+    <t>勾引</t>
+  </si>
+  <si>
+    <t>主动：对手立即再抽1张</t>
+  </si>
+  <si>
+    <t>废土</t>
+  </si>
+  <si>
+    <t>被动：对手队列中每有一张“污染”，则自身+1分</t>
+  </si>
+  <si>
+    <t>毒源</t>
   </si>
   <si>
     <t>被动：在队列中时，对手每再抽一张，就往对手弃牌堆中，加入一张“污染”（具有临时效果，-1分）</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>主动：对手立即再抽1张</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>商店价格</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>主动：复制自己队列中的一张卡，具有临时效果</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>被动：此后抽取的卡获得+1分</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>被动：如果是最后一张，则+3分</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>复制</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>先锋</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>小鬼</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>污染</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>废土</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>毒源</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>圣光</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>主动：使队列中其他卡牌获得+1分</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>莽夫</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>首领</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>ID</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>主动：选择队列中另外一张卡，将其洗回抽牌堆</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>是否解锁</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>被动：被抽取时，会立即再抽2张</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>被动:如果对手的队列数量小于等于3，则自身+2分</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>被动：队列中每有1个分数低于2的卡牌，则自身+1分</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>被动：在队列中时，对手每再抽一张，则自身+1分</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>被动：在队列中时，对手每再抽一张，则自身-1分</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>被动：对手队列中每有一张“污染”，则自身+1分</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>一分</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>三分</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>牌名</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>二分</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>贷款</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>陷阱</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>回收</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>勾引</t>
-  </si>
-  <si>
-    <t>魅魔</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>掀桌</t>
-    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>泄密</t>
   </si>
   <si>
     <t>被动：对手队列中每有1个炸弹，自身+3分</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>泄密</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -278,13 +215,14 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -618,37 +556,37 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6EBCBEC8-5D21-4A68-9874-E023DEBF469A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G23"/>
   <sheetFormatPr defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="3" width="16.3984375" customWidth="1"/>
-    <col min="4" max="4" width="10.46484375" customWidth="1"/>
-    <col min="6" max="6" width="11.86328125" customWidth="1"/>
-    <col min="7" max="7" width="43.53125" customWidth="1"/>
+    <col min="1" max="3" width="16.3984375" style="2" customWidth="1"/>
+    <col min="4" max="4" width="10.46484375" style="2" customWidth="1"/>
+    <col min="6" max="6" width="11.86328125" style="2" customWidth="1"/>
+    <col min="7" max="7" width="43.53125" style="2" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>38</v>
+        <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>29</v>
+        <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="F1" t="s">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G1" t="s">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.4">
@@ -656,7 +594,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>36</v>
+        <v>7</v>
       </c>
       <c r="C2" s="1" t="b">
         <v>1</v>
@@ -673,7 +611,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>39</v>
+        <v>8</v>
       </c>
       <c r="C3" s="1" t="b">
         <v>1</v>
@@ -690,7 +628,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>37</v>
+        <v>9</v>
       </c>
       <c r="C4" s="1" t="b">
         <v>1</v>
@@ -707,7 +645,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>41</v>
+        <v>10</v>
       </c>
       <c r="C5" s="1" t="b">
         <v>1</v>
@@ -719,10 +657,10 @@
         <v>-1</v>
       </c>
       <c r="F5" t="s">
-        <v>41</v>
+        <v>10</v>
       </c>
       <c r="G5" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.4">
@@ -730,7 +668,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="C6" s="1" t="b">
         <v>1</v>
@@ -742,10 +680,10 @@
         <v>1</v>
       </c>
       <c r="F6" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="G6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.4">
@@ -753,7 +691,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="C7" s="1" t="b">
         <v>1</v>
@@ -765,10 +703,10 @@
         <v>5</v>
       </c>
       <c r="F7" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="G7" t="s">
-        <v>30</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.4">
@@ -776,7 +714,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C8" s="1" t="b">
         <v>1</v>
@@ -788,10 +726,10 @@
         <v>1</v>
       </c>
       <c r="F8" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="G8" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.4">
@@ -799,7 +737,7 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C9" s="1" t="b">
         <v>1</v>
@@ -811,10 +749,10 @@
         <v>1</v>
       </c>
       <c r="F9" t="s">
+        <v>18</v>
+      </c>
+      <c r="G9" t="s">
         <v>19</v>
-      </c>
-      <c r="G9" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.4">
@@ -822,7 +760,7 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="C10" s="1" t="b">
         <v>1</v>
@@ -834,10 +772,10 @@
         <v>2</v>
       </c>
       <c r="F10" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="G10" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.4">
@@ -845,7 +783,7 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="C11" s="1" t="b">
         <v>1</v>
@@ -857,10 +795,10 @@
         <v>1</v>
       </c>
       <c r="F11" t="s">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="G11" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.4">
@@ -868,7 +806,7 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C12" s="1" t="b">
         <v>1</v>
@@ -880,10 +818,10 @@
         <v>0</v>
       </c>
       <c r="F12" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="G12" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.4">
@@ -891,7 +829,7 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>2</v>
+        <v>26</v>
       </c>
       <c r="C13" s="1" t="b">
         <v>1</v>
@@ -903,10 +841,10 @@
         <v>0</v>
       </c>
       <c r="F13" t="s">
-        <v>2</v>
+        <v>26</v>
       </c>
       <c r="G13" t="s">
-        <v>4</v>
+        <v>27</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.4">
@@ -914,7 +852,7 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>3</v>
+        <v>28</v>
       </c>
       <c r="C14" s="1" t="b">
         <v>1</v>
@@ -926,10 +864,10 @@
         <v>1</v>
       </c>
       <c r="F14" t="s">
-        <v>3</v>
+        <v>28</v>
       </c>
       <c r="G14" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.4">
@@ -937,7 +875,7 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>6</v>
+        <v>30</v>
       </c>
       <c r="C15" s="1" t="b">
         <v>1</v>
@@ -949,10 +887,10 @@
         <v>0</v>
       </c>
       <c r="F15" t="s">
-        <v>6</v>
+        <v>30</v>
       </c>
       <c r="G15" t="s">
-        <v>5</v>
+        <v>31</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.4">
@@ -960,7 +898,7 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>44</v>
+        <v>32</v>
       </c>
       <c r="C16" s="1" t="b">
         <v>1</v>
@@ -972,7 +910,7 @@
         <v>0</v>
       </c>
       <c r="F16" t="s">
-        <v>44</v>
+        <v>32</v>
       </c>
       <c r="G16" t="s">
         <v>33</v>
@@ -983,7 +921,7 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>45</v>
+        <v>34</v>
       </c>
       <c r="C17" s="1" t="b">
         <v>1</v>
@@ -995,10 +933,10 @@
         <v>0</v>
       </c>
       <c r="F17" t="s">
-        <v>45</v>
+        <v>34</v>
       </c>
       <c r="G17" t="s">
-        <v>9</v>
+        <v>35</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.4">
@@ -1006,7 +944,7 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="C18" s="1" t="b">
         <v>1</v>
@@ -1018,10 +956,10 @@
         <v>1</v>
       </c>
       <c r="F18" t="s">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="G18" t="s">
-        <v>10</v>
+        <v>37</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.4">
@@ -1029,7 +967,7 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C19" s="1" t="b">
         <v>1</v>
@@ -1041,10 +979,10 @@
         <v>4</v>
       </c>
       <c r="F19" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G19" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.4">
@@ -1052,7 +990,7 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="C20" s="1" t="b">
         <v>1</v>
@@ -1064,10 +1002,10 @@
         <v>1</v>
       </c>
       <c r="F20" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="G20" t="s">
-        <v>12</v>
+        <v>41</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.4">
@@ -1075,7 +1013,7 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>21</v>
+        <v>42</v>
       </c>
       <c r="C21" s="1" t="b">
         <v>1</v>
@@ -1087,10 +1025,10 @@
         <v>1</v>
       </c>
       <c r="F21" t="s">
-        <v>21</v>
+        <v>42</v>
       </c>
       <c r="G21" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.4">
@@ -1098,7 +1036,7 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>22</v>
+        <v>44</v>
       </c>
       <c r="C22" s="1" t="b">
         <v>1</v>
@@ -1110,10 +1048,10 @@
         <v>2</v>
       </c>
       <c r="F22" t="s">
-        <v>22</v>
+        <v>44</v>
       </c>
       <c r="G22" t="s">
-        <v>11</v>
+        <v>45</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.4">
@@ -1121,7 +1059,7 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C23" s="1" t="b">
         <v>0</v>
@@ -1133,10 +1071,10 @@
         <v>0</v>
       </c>
       <c r="F23" t="s">
+        <v>46</v>
+      </c>
+      <c r="G23" t="s">
         <v>47</v>
-      </c>
-      <c r="G23" t="s">
-        <v>46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update run rewards and deck data
</commit_message>
<xml_diff>
--- a/Data/carddesign.xlsx
+++ b/Data/carddesign.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\TapMiniGame\CardLoot\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEBABE09-4AD7-490C-A8B6-121558E0EC59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A5731B5-71F8-46B5-9641-C7A19255C8AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -148,9 +148,6 @@
     <t>主动：对手立即再抽1张</t>
   </si>
   <si>
-    <t>废土</t>
-  </si>
-  <si>
     <t>被动：对手队列中每有一张“污染”，则自身+1分</t>
   </si>
   <si>
@@ -164,6 +161,10 @@
   </si>
   <si>
     <t>被动：对手队列中每有1个炸弹，自身+3分</t>
+  </si>
+  <si>
+    <t>毒爆</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -1013,7 +1014,7 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="C21" s="1" t="b">
         <v>1</v>
@@ -1025,10 +1026,10 @@
         <v>1</v>
       </c>
       <c r="F21" t="s">
+        <v>47</v>
+      </c>
+      <c r="G21" t="s">
         <v>42</v>
-      </c>
-      <c r="G21" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.4">
@@ -1036,7 +1037,7 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C22" s="1" t="b">
         <v>1</v>
@@ -1048,10 +1049,10 @@
         <v>2</v>
       </c>
       <c r="F22" t="s">
+        <v>43</v>
+      </c>
+      <c r="G22" t="s">
         <v>44</v>
-      </c>
-      <c r="G22" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.4">
@@ -1059,7 +1060,7 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C23" s="1" t="b">
         <v>0</v>
@@ -1071,10 +1072,10 @@
         <v>0</v>
       </c>
       <c r="F23" t="s">
+        <v>45</v>
+      </c>
+      <c r="G23" t="s">
         <v>46</v>
-      </c>
-      <c r="G23" t="s">
-        <v>47</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Expand card effects and AI deck support
</commit_message>
<xml_diff>
--- a/Data/carddesign.xlsx
+++ b/Data/carddesign.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\TapMiniGame\CardLoot\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A5731B5-71F8-46B5-9641-C7A19255C8AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60E1C475-EE8F-447F-AC95-055380A79239}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="71">
   <si>
     <t>ID</t>
   </si>
@@ -55,24 +55,15 @@
     <t>陷阱</t>
   </si>
   <si>
-    <t>弃置：往对手抽牌堆中放入一枚“临时”炸弹</t>
-  </si>
-  <si>
     <t>复制</t>
   </si>
   <si>
     <t>主动：复制自己队列中的一张卡，具有临时效果</t>
   </si>
   <si>
-    <t>莽夫</t>
-  </si>
-  <si>
     <t>被动：被抽取时，会立即再抽2张</t>
   </si>
   <si>
-    <t>先锋</t>
-  </si>
-  <si>
     <t>被动：此后抽取的卡获得+1分</t>
   </si>
   <si>
@@ -82,9 +73,6 @@
     <t>被动：如果是最后一张，则+3分</t>
   </si>
   <si>
-    <t>圣光</t>
-  </si>
-  <si>
     <t>主动：使队列中其他卡牌获得+1分</t>
   </si>
   <si>
@@ -94,9 +82,6 @@
     <t>主动：选择队列中另外一张卡，将其洗回抽牌堆</t>
   </si>
   <si>
-    <t>首领</t>
-  </si>
-  <si>
     <t>被动：队列中每有1个分数低于2的卡牌，则自身+1分</t>
   </si>
   <si>
@@ -109,9 +94,6 @@
     <t>虚张</t>
   </si>
   <si>
-    <t>被动:如果对手的队列数量小于等于3，则自身+2分</t>
-  </si>
-  <si>
     <t>恐吓</t>
   </si>
   <si>
@@ -164,6 +146,120 @@
   </si>
   <si>
     <t>毒爆</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>弃置：往对手弃牌堆中放入一枚“临时”炸弹</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>被动：该牌获得的所有额外分数翻倍</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>主动：选择队列中另外一张牌，使其+2分</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>被动：每当你抽取一张牌时，与队列随机另一张牌交换位置</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>主动：选择弃牌堆中的一张牌，将其加入队列</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>主动：抽一张牌，如果是炸弹则将其弃置且不会受到伤害</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>换位</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>灵动</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>旗帜</t>
+  </si>
+  <si>
+    <t>旗帜</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>钓钩</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>被动：如果队列被抽满了，则自身+4分</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>被动:   如果对手的队列数量小于等于5，则自身+2分</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>收纳</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>整理</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>争先</t>
+  </si>
+  <si>
+    <t>争先</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>拆除</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>交换</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>心脏</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>手术</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>被动：相邻下一个位置的牌+3分</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>激素</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>主动：选择队列中另一张牌，与其交换位置</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>鲁莽</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>被动：如果是队列第一张牌，则自身+4分</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>筷子</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>被动：被抽取时，在队列中加入一张临时的“一分”</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>购物</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -188,7 +284,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -198,6 +294,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -216,7 +318,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -224,6 +326,12 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -558,7 +666,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="3" width="16.3984375" style="2" customWidth="1"/>
@@ -661,7 +769,7 @@
         <v>10</v>
       </c>
       <c r="G5" t="s">
-        <v>11</v>
+        <v>42</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.4">
@@ -669,7 +777,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C6" s="1" t="b">
         <v>1</v>
@@ -681,10 +789,10 @@
         <v>1</v>
       </c>
       <c r="F6" t="s">
+        <v>11</v>
+      </c>
+      <c r="G6" t="s">
         <v>12</v>
-      </c>
-      <c r="G6" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.4">
@@ -692,7 +800,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>14</v>
+        <v>66</v>
       </c>
       <c r="C7" s="1" t="b">
         <v>1</v>
@@ -704,10 +812,10 @@
         <v>5</v>
       </c>
       <c r="F7" t="s">
-        <v>14</v>
+        <v>66</v>
       </c>
       <c r="G7" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.4">
@@ -715,7 +823,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>16</v>
+        <v>50</v>
       </c>
       <c r="C8" s="1" t="b">
         <v>1</v>
@@ -727,10 +835,10 @@
         <v>1</v>
       </c>
       <c r="F8" t="s">
-        <v>16</v>
+        <v>51</v>
       </c>
       <c r="G8" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.4">
@@ -738,7 +846,7 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="C9" s="1" t="b">
         <v>1</v>
@@ -750,10 +858,10 @@
         <v>1</v>
       </c>
       <c r="F9" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="G9" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.4">
@@ -761,22 +869,22 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>20</v>
-      </c>
-      <c r="C10" s="1" t="b">
+        <v>56</v>
+      </c>
+      <c r="C10" s="3" t="b">
         <v>1</v>
       </c>
       <c r="D10">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="E10">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F10" t="s">
-        <v>20</v>
+        <v>56</v>
       </c>
       <c r="G10" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.4">
@@ -784,7 +892,7 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="C11" s="1" t="b">
         <v>1</v>
@@ -796,10 +904,10 @@
         <v>1</v>
       </c>
       <c r="F11" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="G11" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.4">
@@ -807,22 +915,22 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>24</v>
-      </c>
-      <c r="C12" s="1" t="b">
+        <v>55</v>
+      </c>
+      <c r="C12" s="3" t="b">
         <v>1</v>
       </c>
       <c r="D12">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E12">
         <v>0</v>
       </c>
       <c r="F12" t="s">
-        <v>24</v>
+        <v>55</v>
       </c>
       <c r="G12" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.4">
@@ -830,7 +938,7 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="C13" s="1" t="b">
         <v>1</v>
@@ -842,10 +950,10 @@
         <v>0</v>
       </c>
       <c r="F13" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="G13" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.4">
@@ -853,9 +961,9 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>28</v>
-      </c>
-      <c r="C14" s="1" t="b">
+        <v>23</v>
+      </c>
+      <c r="C14" s="3" t="b">
         <v>1</v>
       </c>
       <c r="D14">
@@ -865,10 +973,10 @@
         <v>1</v>
       </c>
       <c r="F14" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="G14" t="s">
-        <v>29</v>
+        <v>54</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.4">
@@ -876,7 +984,7 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="C15" s="1" t="b">
         <v>1</v>
@@ -888,10 +996,10 @@
         <v>0</v>
       </c>
       <c r="F15" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="G15" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.4">
@@ -899,7 +1007,7 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="C16" s="1" t="b">
         <v>1</v>
@@ -911,10 +1019,10 @@
         <v>0</v>
       </c>
       <c r="F16" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="G16" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.4">
@@ -922,7 +1030,7 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="C17" s="1" t="b">
         <v>1</v>
@@ -934,10 +1042,10 @@
         <v>0</v>
       </c>
       <c r="F17" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="G17" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.4">
@@ -945,7 +1053,7 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="C18" s="1" t="b">
         <v>1</v>
@@ -957,10 +1065,10 @@
         <v>1</v>
       </c>
       <c r="F18" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="G18" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.4">
@@ -968,7 +1076,7 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="C19" s="1" t="b">
         <v>1</v>
@@ -980,10 +1088,10 @@
         <v>4</v>
       </c>
       <c r="F19" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="G19" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.4">
@@ -991,7 +1099,7 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="C20" s="1" t="b">
         <v>1</v>
@@ -1003,10 +1111,10 @@
         <v>1</v>
       </c>
       <c r="F20" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="G20" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.4">
@@ -1014,7 +1122,7 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="C21" s="1" t="b">
         <v>1</v>
@@ -1026,10 +1134,10 @@
         <v>1</v>
       </c>
       <c r="F21" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="G21" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.4">
@@ -1037,22 +1145,22 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="C22" s="1" t="b">
         <v>1</v>
       </c>
       <c r="D22">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E22">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F22" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="G22" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.4">
@@ -1060,10 +1168,10 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="C23" s="1" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D23">
         <v>8</v>
@@ -1072,10 +1180,240 @@
         <v>0</v>
       </c>
       <c r="F23" t="s">
+        <v>39</v>
+      </c>
+      <c r="G23" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A24" s="1">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C24" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="D24" s="2">
+        <v>5</v>
+      </c>
+      <c r="E24">
+        <v>1</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A25" s="1">
+        <v>24</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C25" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="D25" s="2">
+        <v>6</v>
+      </c>
+      <c r="E25">
+        <v>1</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A26" s="1">
+        <v>25</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C26" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="D26" s="2">
+        <v>8</v>
+      </c>
+      <c r="E26">
+        <v>0</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A27" s="1">
+        <v>26</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C27" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="D27" s="2">
+        <v>6</v>
+      </c>
+      <c r="E27">
+        <v>1</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="G27" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A28" s="1">
+        <v>27</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C28" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="D28" s="2">
+        <v>4</v>
+      </c>
+      <c r="E28">
+        <v>1</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A29" s="1">
+        <v>28</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C29" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="D29" s="2">
+        <v>5</v>
+      </c>
+      <c r="E29">
+        <v>2</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="G29" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="G23" t="s">
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A30" s="1">
+        <v>29</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C30" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="D30" s="2">
+        <v>5</v>
+      </c>
+      <c r="E30">
+        <v>1</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A31" s="1">
+        <v>30</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C31" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="D31" s="2">
+        <v>4</v>
+      </c>
+      <c r="E31">
+        <v>0</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="G31" s="2" t="s">
         <v>46</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A32" s="1">
+        <v>31</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C32" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="D32" s="2">
+        <v>6</v>
+      </c>
+      <c r="E32">
+        <v>1</v>
+      </c>
+      <c r="F32" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="G32" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A33" s="4">
+        <v>32</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C33" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="D33" s="2">
+        <v>4</v>
+      </c>
+      <c r="E33">
+        <v>1</v>
+      </c>
+      <c r="F33" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="G33" s="2" t="s">
+        <v>69</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Expand special card systems
</commit_message>
<xml_diff>
--- a/Data/carddesign.xlsx
+++ b/Data/carddesign.xlsx
@@ -8,19 +8,34 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\TapMiniGame\CardLoot\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60E1C475-EE8F-447F-AC95-055380A79239}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E772ECA-1B04-430C-BE26-5513C6B16E9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="全卡表" sheetId="1" r:id="rId1"/>
+    <sheet name="负面卡表" sheetId="2" r:id="rId2"/>
+    <sheet name="特殊卡表" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="103">
   <si>
     <t>ID</t>
   </si>
@@ -52,9 +67,6 @@
     <t>三分</t>
   </si>
   <si>
-    <t>陷阱</t>
-  </si>
-  <si>
     <t>复制</t>
   </si>
   <si>
@@ -76,9 +88,6 @@
     <t>主动：使队列中其他卡牌获得+1分</t>
   </si>
   <si>
-    <t>回收</t>
-  </si>
-  <si>
     <t>主动：选择队列中另外一张卡，将其洗回抽牌堆</t>
   </si>
   <si>
@@ -139,20 +148,10 @@
     <t>被动：在队列中时，对手每再抽一张，就往对手弃牌堆中，加入一张“污染”（具有临时效果，-1分）</t>
   </si>
   <si>
-    <t>泄密</t>
-  </si>
-  <si>
-    <t>被动：对手队列中每有1个炸弹，自身+3分</t>
-  </si>
-  <si>
     <t>毒爆</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>弃置：往对手弃牌堆中放入一枚“临时”炸弹</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>被动：该牌获得的所有额外分数翻倍</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -169,10 +168,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>主动：抽一张牌，如果是炸弹则将其弃置且不会受到伤害</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>换位</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -215,10 +210,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>拆除</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>交换</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -260,6 +251,160 @@
   </si>
   <si>
     <t>购物</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>负二</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>被动：每再抽1张，则自身-1分</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>腐蚀</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>封禁</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>被动：抽到时，立即停牌</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>被动：抽到炸弹时，额外扣除1点阈值</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>火药</t>
+  </si>
+  <si>
+    <t>火药</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>神像</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>自身分数等于对手队列中分数最高的</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>弃置：往对手弃牌堆中放入一张“临时”炸弹</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>埋伏</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>主动：双方均扣除1点阈值点</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>威胁</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>主动：对方立即将弃牌堆洗回抽牌堆</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>冷静</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>被动：每当被抽取时，回复1点阈值点</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>自爆</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>被动：对手队列中每有1个炸弹，自身+2分</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>大鱼</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>打捞</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>主动：将你的弃牌堆立即洗回抽牌堆</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>被动：如果是从弃牌堆进入队列，则自身+3分</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>小鱼</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>被动：每次进入弃牌堆，本局期间+2分</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>抢单</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>主动：立即再抽2张，然后自身+2分</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>差评</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>主动：选择对手队列中一张卡，使其分数减半（向下取整）</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>外卖</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>被动：抽取时，往对手队列中中加入一张临时的1分</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>断点</t>
+  </si>
+  <si>
+    <t>断点</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>回滚</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>主动：抽一张牌并立即将其弃掉，如果是炸弹不会受到伤害</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>假货</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>劣币</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>被动：队列中每有一张劣币，自身+1分</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>被动：每次进入弃牌堆，本局期间-2分</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -666,7 +811,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:G44"/>
   <sheetFormatPr defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="3" width="16.3984375" style="2" customWidth="1"/>
@@ -754,7 +899,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>10</v>
+        <v>75</v>
       </c>
       <c r="C5" s="1" t="b">
         <v>1</v>
@@ -766,10 +911,10 @@
         <v>-1</v>
       </c>
       <c r="F5" t="s">
-        <v>10</v>
+        <v>75</v>
       </c>
       <c r="G5" t="s">
-        <v>42</v>
+        <v>74</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.4">
@@ -777,7 +922,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C6" s="1" t="b">
         <v>1</v>
@@ -789,10 +934,10 @@
         <v>1</v>
       </c>
       <c r="F6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G6" t="s">
         <v>11</v>
-      </c>
-      <c r="G6" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.4">
@@ -800,7 +945,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="C7" s="1" t="b">
         <v>1</v>
@@ -812,10 +957,10 @@
         <v>5</v>
       </c>
       <c r="F7" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="G7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.4">
@@ -823,7 +968,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="C8" s="1" t="b">
         <v>1</v>
@@ -835,10 +980,10 @@
         <v>1</v>
       </c>
       <c r="F8" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="G8" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.4">
@@ -846,7 +991,7 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C9" s="1" t="b">
         <v>1</v>
@@ -858,10 +1003,10 @@
         <v>1</v>
       </c>
       <c r="F9" t="s">
+        <v>14</v>
+      </c>
+      <c r="G9" t="s">
         <v>15</v>
-      </c>
-      <c r="G9" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.4">
@@ -869,7 +1014,7 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="C10" s="3" t="b">
         <v>1</v>
@@ -881,10 +1026,10 @@
         <v>0</v>
       </c>
       <c r="F10" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="G10" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.4">
@@ -892,7 +1037,7 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>18</v>
+        <v>97</v>
       </c>
       <c r="C11" s="1" t="b">
         <v>1</v>
@@ -904,10 +1049,10 @@
         <v>1</v>
       </c>
       <c r="F11" t="s">
-        <v>18</v>
+        <v>97</v>
       </c>
       <c r="G11" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.4">
@@ -915,7 +1060,7 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="C12" s="3" t="b">
         <v>1</v>
@@ -927,10 +1072,10 @@
         <v>0</v>
       </c>
       <c r="F12" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="G12" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.4">
@@ -938,7 +1083,7 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C13" s="1" t="b">
         <v>1</v>
@@ -950,10 +1095,10 @@
         <v>0</v>
       </c>
       <c r="F13" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="G13" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.4">
@@ -961,7 +1106,7 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C14" s="3" t="b">
         <v>1</v>
@@ -973,10 +1118,10 @@
         <v>1</v>
       </c>
       <c r="F14" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="G14" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.4">
@@ -984,7 +1129,7 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C15" s="1" t="b">
         <v>1</v>
@@ -996,10 +1141,10 @@
         <v>0</v>
       </c>
       <c r="F15" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="G15" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.4">
@@ -1007,7 +1152,7 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C16" s="1" t="b">
         <v>1</v>
@@ -1019,10 +1164,10 @@
         <v>0</v>
       </c>
       <c r="F16" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="G16" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.4">
@@ -1030,7 +1175,7 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C17" s="1" t="b">
         <v>1</v>
@@ -1042,10 +1187,10 @@
         <v>0</v>
       </c>
       <c r="F17" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="G17" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.4">
@@ -1053,7 +1198,7 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C18" s="1" t="b">
         <v>1</v>
@@ -1065,10 +1210,10 @@
         <v>1</v>
       </c>
       <c r="F18" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="G18" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.4">
@@ -1076,7 +1221,7 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C19" s="1" t="b">
         <v>1</v>
@@ -1088,10 +1233,10 @@
         <v>4</v>
       </c>
       <c r="F19" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="G19" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.4">
@@ -1099,7 +1244,7 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C20" s="1" t="b">
         <v>1</v>
@@ -1111,10 +1256,10 @@
         <v>1</v>
       </c>
       <c r="F20" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="G20" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.4">
@@ -1122,7 +1267,7 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C21" s="1" t="b">
         <v>1</v>
@@ -1134,10 +1279,10 @@
         <v>1</v>
       </c>
       <c r="F21" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="G21" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.4">
@@ -1145,7 +1290,7 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C22" s="1" t="b">
         <v>1</v>
@@ -1157,10 +1302,10 @@
         <v>0</v>
       </c>
       <c r="F22" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="G22" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.4">
@@ -1168,22 +1313,22 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>39</v>
+        <v>71</v>
       </c>
       <c r="C23" s="1" t="b">
         <v>1</v>
       </c>
       <c r="D23">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E23">
         <v>0</v>
       </c>
       <c r="F23" t="s">
-        <v>39</v>
+        <v>71</v>
       </c>
       <c r="G23" t="s">
-        <v>40</v>
+        <v>82</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.4">
@@ -1191,7 +1336,7 @@
         <v>23</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="C24" s="1" t="b">
         <v>1</v>
@@ -1203,10 +1348,10 @@
         <v>1</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.4">
@@ -1214,7 +1359,7 @@
         <v>24</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="C25" s="1" t="b">
         <v>1</v>
@@ -1226,10 +1371,10 @@
         <v>1</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.4">
@@ -1237,7 +1382,7 @@
         <v>25</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="C26" s="1" t="b">
         <v>1</v>
@@ -1249,10 +1394,10 @@
         <v>0</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.4">
@@ -1260,7 +1405,7 @@
         <v>26</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="C27" s="1" t="b">
         <v>1</v>
@@ -1272,10 +1417,10 @@
         <v>1</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.4">
@@ -1283,7 +1428,7 @@
         <v>27</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="C28" s="1" t="b">
         <v>1</v>
@@ -1295,10 +1440,10 @@
         <v>1</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.4">
@@ -1306,7 +1451,7 @@
         <v>28</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="C29" s="1" t="b">
         <v>1</v>
@@ -1318,10 +1463,10 @@
         <v>2</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.4">
@@ -1329,7 +1474,7 @@
         <v>29</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="C30" s="1" t="b">
         <v>1</v>
@@ -1341,10 +1486,10 @@
         <v>1</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.4">
@@ -1352,7 +1497,7 @@
         <v>30</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="C31" s="1" t="b">
         <v>1</v>
@@ -1364,10 +1509,10 @@
         <v>0</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.4">
@@ -1375,30 +1520,30 @@
         <v>31</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>59</v>
+        <v>95</v>
       </c>
       <c r="C32" s="1" t="b">
         <v>1</v>
       </c>
       <c r="D32" s="2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E32">
         <v>1</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>59</v>
+        <v>96</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>47</v>
+        <v>98</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A33" s="4">
+      <c r="A33" s="1">
         <v>32</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="C33" s="1" t="b">
         <v>1</v>
@@ -1410,10 +1555,407 @@
         <v>1</v>
       </c>
       <c r="F33" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="G33" s="2" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A34" s="1">
+        <v>33</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C34" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="D34" s="2">
+        <v>5</v>
+      </c>
+      <c r="E34">
+        <v>0</v>
+      </c>
+      <c r="F34" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="G34" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A35" s="1">
+        <v>34</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C35" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="D35" s="2">
+        <v>5</v>
+      </c>
+      <c r="E35">
+        <v>0</v>
+      </c>
+      <c r="F35" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="G35" s="2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A36" s="1">
+        <v>35</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C36" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="D36" s="2">
+        <v>6</v>
+      </c>
+      <c r="E36">
+        <v>-3</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="G36" s="2" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A37" s="4">
+        <v>36</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C37" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="D37" s="2">
+        <v>6</v>
+      </c>
+      <c r="E37">
+        <v>2</v>
+      </c>
+      <c r="F37" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="G37" s="2" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A38" s="4">
+        <v>37</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="C38" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="D38" s="2">
+        <v>6</v>
+      </c>
+      <c r="E38">
+        <v>0</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="G38" s="2" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A39" s="4">
+        <v>38</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C39" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="D39" s="2">
+        <v>7</v>
+      </c>
+      <c r="E39">
+        <v>2</v>
+      </c>
+      <c r="F39" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="G39" s="2" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A40" s="4">
+        <v>39</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="C40" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="D40" s="2">
+        <v>6</v>
+      </c>
+      <c r="E40">
+        <v>2</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="G40" s="2" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A41" s="4">
+        <v>40</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="C41" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="D41" s="2">
+        <v>5</v>
+      </c>
+      <c r="E41">
+        <v>1</v>
+      </c>
+      <c r="F41" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="G41" s="2" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A42" s="4">
+        <v>41</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="C42" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="D42" s="2">
+        <v>3</v>
+      </c>
+      <c r="E42">
+        <v>2</v>
+      </c>
+      <c r="F42" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="G42" s="2" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A43" s="4">
+        <v>42</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="C43" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="D43" s="2">
+        <v>3</v>
+      </c>
+      <c r="E43">
+        <v>0</v>
+      </c>
+      <c r="F43" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="G43" s="2" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A44" s="4">
+        <v>43</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="C44" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="D44" s="2">
+        <v>6</v>
+      </c>
+      <c r="E44">
+        <v>6</v>
+      </c>
+      <c r="F44" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="G44" s="2" t="s">
+        <v>102</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B1E4554-1D79-4299-B118-A232D22D8BFA}">
+  <dimension ref="A1:E5"/>
+  <sheetFormatPr defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="3" max="3" width="10.59765625" customWidth="1"/>
+    <col min="4" max="4" width="12.6640625" customWidth="1"/>
+    <col min="5" max="5" width="39.796875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C2">
+        <v>-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>66</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+      <c r="D3" t="s">
+        <v>66</v>
+      </c>
+      <c r="E3" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>67</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4" t="s">
+        <v>67</v>
+      </c>
+      <c r="E4" t="s">
         <v>68</v>
       </c>
-      <c r="G33" s="2" t="s">
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>70</v>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+      <c r="D5" t="s">
+        <v>71</v>
+      </c>
+      <c r="E5" t="s">
         <v>69</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B2D8529-B1E2-4EBC-832A-281508D7A10D}">
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="4" max="4" width="10" customWidth="1"/>
+    <col min="5" max="5" width="38.1328125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>72</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+      <c r="D2" t="s">
+        <v>72</v>
+      </c>
+      <c r="E2" t="s">
+        <v>73</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add catalog progression and late-game cards
</commit_message>
<xml_diff>
--- a/Data/carddesign.xlsx
+++ b/Data/carddesign.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\TapMiniGame\CardLoot\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E772ECA-1B04-430C-BE26-5513C6B16E9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE39E8CA-DAC1-4C1F-963A-446DCF01ECA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-285" yWindow="165" windowWidth="14400" windowHeight="9840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="全卡表" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="128">
   <si>
     <t>ID</t>
   </si>
@@ -70,341 +70,444 @@
     <t>复制</t>
   </si>
   <si>
+    <t>被动：被抽取时，会立即再抽2张</t>
+  </si>
+  <si>
+    <t>被动：此后抽取的卡获得+1分</t>
+  </si>
+  <si>
+    <t>小鬼</t>
+  </si>
+  <si>
+    <t>被动：如果是最后一张，则+3分</t>
+  </si>
+  <si>
+    <t>主动：使队列中其他卡牌获得+1分</t>
+  </si>
+  <si>
+    <t>主动：选择队列中另外一张卡，将其洗回抽牌堆</t>
+  </si>
+  <si>
+    <t>被动：队列中每有1个分数低于2的卡牌，则自身+1分</t>
+  </si>
+  <si>
+    <t>偷窃</t>
+  </si>
+  <si>
+    <t>虚张</t>
+  </si>
+  <si>
+    <t>恐吓</t>
+  </si>
+  <si>
+    <t>主动：随机弃掉对手队列中的一个卡</t>
+  </si>
+  <si>
+    <t>魅魔</t>
+  </si>
+  <si>
+    <t>被动：在队列中时，对手每再抽一张，则自身+1分</t>
+  </si>
+  <si>
+    <t>掀桌</t>
+  </si>
+  <si>
+    <t>主动：双方各随机弃2张牌</t>
+  </si>
+  <si>
+    <t>污染</t>
+  </si>
+  <si>
+    <t>主动：往对手弃牌堆中，加入一张“污染”（具有临时效果，-1分）</t>
+  </si>
+  <si>
+    <t>贷款</t>
+  </si>
+  <si>
+    <t>被动：在队列中时，对手每再抽一张，则自身-1分</t>
+  </si>
+  <si>
+    <t>勾引</t>
+  </si>
+  <si>
+    <t>主动：对手立即再抽1张</t>
+  </si>
+  <si>
+    <t>被动：对手队列中每有一张“污染”，则自身+1分</t>
+  </si>
+  <si>
+    <t>毒源</t>
+  </si>
+  <si>
+    <t>被动：在队列中时，对手每再抽一张，就往对手弃牌堆中，加入一张“污染”（具有临时效果，-1分）</t>
+  </si>
+  <si>
+    <t>毒爆</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>被动：该牌获得的所有额外分数翻倍</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>主动：选择队列中另外一张牌，使其+2分</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>被动：每当你抽取一张牌时，与队列随机另一张牌交换位置</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>主动：选择弃牌堆中的一张牌，将其加入队列</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>换位</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>灵动</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>旗帜</t>
+  </si>
+  <si>
+    <t>旗帜</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>钓钩</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>被动：如果队列被抽满了，则自身+4分</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>被动:   如果对手的队列数量小于等于5，则自身+2分</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>收纳</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>整理</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>争先</t>
+  </si>
+  <si>
+    <t>争先</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>交换</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>心脏</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>手术</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>被动：相邻下一个位置的牌+3分</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>激素</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>主动：选择队列中另一张牌，与其交换位置</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>鲁莽</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>被动：如果是队列第一张牌，则自身+4分</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>筷子</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>被动：被抽取时，在队列中加入一张临时的“一分”</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>购物</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>负二</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>腐蚀</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>封禁</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>被动：抽到时，立即停牌</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>被动：抽到炸弹时，额外扣除1点阈值</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>火药</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>神像</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>自身分数等于对手队列中分数最高的</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>弃置：往对手弃牌堆中放入一张“临时”炸弹</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>埋伏</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>主动：双方均扣除1点阈值点</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>威胁</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>主动：对方立即将弃牌堆洗回抽牌堆</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>自爆</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>大鱼</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>打捞</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>主动：将你的弃牌堆立即洗回抽牌堆</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>被动：如果是从弃牌堆进入队列，则自身+3分</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>被动：每次进入弃牌堆，本局期间+2分</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>抢单</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>主动：立即再抽2张，然后自身+2分</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>差评</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>主动：选择对手队列中一张卡，使其分数减半（向下取整）</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>外卖</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>被动：抽取时，往对手队列中中加入一张临时的1分</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>断点</t>
+  </si>
+  <si>
+    <t>断点</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>主动：抽一张牌并立即将其弃掉，如果是炸弹不会受到伤害</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>假货</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>劣币</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>被动：队列中每有一张劣币，自身+1分</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>被动：每次进入弃牌堆，本局期间-2分</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>水军</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>主动：往对手弃牌堆中放入两张临时的“零分”</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>榜一</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>被动：如果是双方队列中分数最高的卡，则自身+4分</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>控评</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>主动：随机使对手队列中两张卡-1分</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>求和</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>被动：分数增加相邻的两张卡的分数之和</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>主动：选择队列中一张牌弃掉，自身增加被弃掉牌的分数</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>合并</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>翻倍</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>主动：选择队列中一张牌，使其增加其当前分数</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>狮子</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>主动：选择对手队列中的一张牌，将其弃置</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>犀牛</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>被动：与该卡同一行的卡，获得+1分</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>兽王</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>被动：队列中每有一张不同的动物卡，就获得+2分</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>鹦鹉</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>主动：选择队列中另外一张卡，变为它的复制（进入弃牌堆后恢复）</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>斑马</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>被动：每进行一次抽取，自身分数在1和3之间交替变化</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
     <t>主动：复制自己队列中的一张卡，具有临时效果</t>
-  </si>
-  <si>
-    <t>被动：被抽取时，会立即再抽2张</t>
-  </si>
-  <si>
-    <t>被动：此后抽取的卡获得+1分</t>
-  </si>
-  <si>
-    <t>小鬼</t>
-  </si>
-  <si>
-    <t>被动：如果是最后一张，则+3分</t>
-  </si>
-  <si>
-    <t>主动：使队列中其他卡牌获得+1分</t>
-  </si>
-  <si>
-    <t>主动：选择队列中另外一张卡，将其洗回抽牌堆</t>
-  </si>
-  <si>
-    <t>被动：队列中每有1个分数低于2的卡牌，则自身+1分</t>
-  </si>
-  <si>
-    <t>偷窃</t>
-  </si>
-  <si>
-    <t>主动：选择对手队列中的一个卡，将其放入自身的队列（弃牌后返回对手弃牌堆）</t>
-  </si>
-  <si>
-    <t>虚张</t>
-  </si>
-  <si>
-    <t>恐吓</t>
-  </si>
-  <si>
-    <t>主动：随机弃掉对手队列中的一个卡</t>
-  </si>
-  <si>
-    <t>魅魔</t>
-  </si>
-  <si>
-    <t>被动：在队列中时，对手每再抽一张，则自身+1分</t>
-  </si>
-  <si>
-    <t>掀桌</t>
-  </si>
-  <si>
-    <t>主动：双方各随机弃2张牌</t>
-  </si>
-  <si>
-    <t>污染</t>
-  </si>
-  <si>
-    <t>主动：往对手弃牌堆中，加入一张“污染”（具有临时效果，-1分）</t>
-  </si>
-  <si>
-    <t>贷款</t>
-  </si>
-  <si>
-    <t>被动：在队列中时，对手每再抽一张，则自身-1分</t>
-  </si>
-  <si>
-    <t>勾引</t>
-  </si>
-  <si>
-    <t>主动：对手立即再抽1张</t>
-  </si>
-  <si>
-    <t>被动：对手队列中每有一张“污染”，则自身+1分</t>
-  </si>
-  <si>
-    <t>毒源</t>
-  </si>
-  <si>
-    <t>被动：在队列中时，对手每再抽一张，就往对手弃牌堆中，加入一张“污染”（具有临时效果，-1分）</t>
-  </si>
-  <si>
-    <t>毒爆</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>被动：该牌获得的所有额外分数翻倍</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>主动：选择队列中另外一张牌，使其+2分</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>被动：每当你抽取一张牌时，与队列随机另一张牌交换位置</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>主动：选择弃牌堆中的一张牌，将其加入队列</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>换位</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>灵动</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>旗帜</t>
-  </si>
-  <si>
-    <t>旗帜</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>钓钩</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>被动：如果队列被抽满了，则自身+4分</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>被动:   如果对手的队列数量小于等于5，则自身+2分</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>收纳</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>整理</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>争先</t>
-  </si>
-  <si>
-    <t>争先</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>交换</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>心脏</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>手术</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>被动：相邻下一个位置的牌+3分</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>激素</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>主动：选择队列中另一张牌，与其交换位置</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>鲁莽</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>被动：如果是队列第一张牌，则自身+4分</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>筷子</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>被动：被抽取时，在队列中加入一张临时的“一分”</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>购物</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>负二</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>被动：每再抽1张，则自身-1分</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>腐蚀</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>封禁</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>被动：抽到时，立即停牌</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>被动：抽到炸弹时，额外扣除1点阈值</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>火药</t>
-  </si>
-  <si>
-    <t>火药</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>神像</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>自身分数等于对手队列中分数最高的</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>弃置：往对手弃牌堆中放入一张“临时”炸弹</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>埋伏</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>主动：双方均扣除1点阈值点</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>威胁</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>主动：对方立即将弃牌堆洗回抽牌堆</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>冷静</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>被动：每当被抽取时，回复1点阈值点</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>自爆</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>被动：对手队列中每有1个炸弹，自身+2分</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>大鱼</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>打捞</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>主动：将你的弃牌堆立即洗回抽牌堆</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>被动：如果是从弃牌堆进入队列，则自身+3分</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>小鱼</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>被动：每次进入弃牌堆，本局期间+2分</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>抢单</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>主动：立即再抽2张，然后自身+2分</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>差评</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>主动：选择对手队列中一张卡，使其分数减半（向下取整）</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>外卖</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>被动：抽取时，往对手队列中中加入一张临时的1分</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>断点</t>
-  </si>
-  <si>
-    <t>断点</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>回滚</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>主动：抽一张牌并立即将其弃掉，如果是炸弹不会受到伤害</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>假货</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>劣币</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>被动：队列中每有一张劣币，自身+1分</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>被动：每次进入弃牌堆，本局期间-2分</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>复制</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>螃蟹</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>主动：随机偷取对手队列中的一个卡，将其放入自身的队列（弃牌后返回对手弃牌堆）</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>被动：每当对手失去1点阈值时，自身+3分</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>易伤</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>被动：抽到时，随机弃掉你的另外一张牌</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>回收</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>日志</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>被动：每当有牌离开队列，则自身+2分</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>冥想</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>主动：立即停牌，并回复1点阈值</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -811,7 +914,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G44"/>
+  <dimension ref="A1:G56"/>
   <sheetFormatPr defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="3" width="16.3984375" style="2" customWidth="1"/>
@@ -899,7 +1002,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="C5" s="1" t="b">
         <v>1</v>
@@ -908,13 +1011,13 @@
         <v>5</v>
       </c>
       <c r="E5">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="F5" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="G5" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.4">
@@ -934,10 +1037,10 @@
         <v>1</v>
       </c>
       <c r="F6" t="s">
-        <v>10</v>
+        <v>117</v>
       </c>
       <c r="G6" t="s">
-        <v>11</v>
+        <v>116</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.4">
@@ -945,7 +1048,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C7" s="1" t="b">
         <v>1</v>
@@ -957,10 +1060,10 @@
         <v>5</v>
       </c>
       <c r="F7" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="G7" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.4">
@@ -968,7 +1071,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C8" s="1" t="b">
         <v>1</v>
@@ -980,10 +1083,10 @@
         <v>1</v>
       </c>
       <c r="F8" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="G8" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.4">
@@ -991,7 +1094,7 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C9" s="1" t="b">
         <v>1</v>
@@ -1003,10 +1106,10 @@
         <v>1</v>
       </c>
       <c r="F9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G9" t="s">
         <v>14</v>
-      </c>
-      <c r="G9" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.4">
@@ -1014,7 +1117,7 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C10" s="3" t="b">
         <v>1</v>
@@ -1026,10 +1129,10 @@
         <v>0</v>
       </c>
       <c r="F10" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="G10" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.4">
@@ -1037,7 +1140,7 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>97</v>
+        <v>123</v>
       </c>
       <c r="C11" s="1" t="b">
         <v>1</v>
@@ -1049,10 +1152,10 @@
         <v>1</v>
       </c>
       <c r="F11" t="s">
-        <v>97</v>
+        <v>123</v>
       </c>
       <c r="G11" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.4">
@@ -1060,7 +1163,7 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C12" s="3" t="b">
         <v>1</v>
@@ -1072,10 +1175,10 @@
         <v>0</v>
       </c>
       <c r="F12" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="G12" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.4">
@@ -1083,7 +1186,7 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C13" s="1" t="b">
         <v>1</v>
@@ -1095,10 +1198,10 @@
         <v>0</v>
       </c>
       <c r="F13" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G13" t="s">
-        <v>20</v>
+        <v>119</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.4">
@@ -1106,7 +1209,7 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C14" s="3" t="b">
         <v>1</v>
@@ -1118,10 +1221,10 @@
         <v>1</v>
       </c>
       <c r="F14" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="G14" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.4">
@@ -1129,7 +1232,7 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C15" s="1" t="b">
         <v>1</v>
@@ -1141,10 +1244,10 @@
         <v>0</v>
       </c>
       <c r="F15" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="G15" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.4">
@@ -1152,7 +1255,7 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C16" s="1" t="b">
         <v>1</v>
@@ -1164,10 +1267,10 @@
         <v>0</v>
       </c>
       <c r="F16" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="G16" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.4">
@@ -1175,7 +1278,7 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C17" s="1" t="b">
         <v>1</v>
@@ -1187,10 +1290,10 @@
         <v>0</v>
       </c>
       <c r="F17" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="G17" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.4">
@@ -1198,7 +1301,7 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C18" s="1" t="b">
         <v>1</v>
@@ -1210,10 +1313,10 @@
         <v>1</v>
       </c>
       <c r="F18" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="G18" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.4">
@@ -1221,22 +1324,22 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C19" s="1" t="b">
         <v>1</v>
       </c>
       <c r="D19">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E19">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F19" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="G19" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.4">
@@ -1244,7 +1347,7 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C20" s="1" t="b">
         <v>1</v>
@@ -1256,10 +1359,10 @@
         <v>1</v>
       </c>
       <c r="F20" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="G20" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.4">
@@ -1267,7 +1370,7 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C21" s="1" t="b">
         <v>1</v>
@@ -1279,10 +1382,10 @@
         <v>1</v>
       </c>
       <c r="F21" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="G21" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.4">
@@ -1290,7 +1393,7 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C22" s="1" t="b">
         <v>1</v>
@@ -1302,10 +1405,10 @@
         <v>0</v>
       </c>
       <c r="F22" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="G22" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.4">
@@ -1313,7 +1416,7 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="C23" s="1" t="b">
         <v>1</v>
@@ -1325,10 +1428,10 @@
         <v>0</v>
       </c>
       <c r="F23" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="G23" t="s">
-        <v>82</v>
+        <v>120</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.4">
@@ -1336,7 +1439,7 @@
         <v>23</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C24" s="1" t="b">
         <v>1</v>
@@ -1348,10 +1451,10 @@
         <v>1</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.4">
@@ -1359,7 +1462,7 @@
         <v>24</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C25" s="1" t="b">
         <v>1</v>
@@ -1371,10 +1474,10 @@
         <v>1</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.4">
@@ -1382,7 +1485,7 @@
         <v>25</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C26" s="1" t="b">
         <v>1</v>
@@ -1394,10 +1497,10 @@
         <v>0</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.4">
@@ -1405,7 +1508,7 @@
         <v>26</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C27" s="1" t="b">
         <v>1</v>
@@ -1417,10 +1520,10 @@
         <v>1</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.4">
@@ -1428,7 +1531,7 @@
         <v>27</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C28" s="1" t="b">
         <v>1</v>
@@ -1440,10 +1543,10 @@
         <v>1</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.4">
@@ -1451,7 +1554,7 @@
         <v>28</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C29" s="1" t="b">
         <v>1</v>
@@ -1463,10 +1566,10 @@
         <v>2</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.4">
@@ -1474,7 +1577,7 @@
         <v>29</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C30" s="1" t="b">
         <v>1</v>
@@ -1486,10 +1589,10 @@
         <v>1</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.4">
@@ -1497,7 +1600,7 @@
         <v>30</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C31" s="1" t="b">
         <v>1</v>
@@ -1509,10 +1612,10 @@
         <v>0</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.4">
@@ -1520,7 +1623,7 @@
         <v>31</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="C32" s="1" t="b">
         <v>1</v>
@@ -1532,10 +1635,10 @@
         <v>1</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>98</v>
+        <v>89</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.4">
@@ -1543,7 +1646,7 @@
         <v>32</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C33" s="1" t="b">
         <v>1</v>
@@ -1555,10 +1658,10 @@
         <v>1</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="G33" s="2" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.4">
@@ -1566,7 +1669,7 @@
         <v>33</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="C34" s="1" t="b">
         <v>1</v>
@@ -1578,10 +1681,10 @@
         <v>0</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="G34" s="2" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.4">
@@ -1589,7 +1692,7 @@
         <v>34</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="C35" s="1" t="b">
         <v>1</v>
@@ -1601,10 +1704,10 @@
         <v>0</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="G35" s="2" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.4">
@@ -1612,7 +1715,7 @@
         <v>35</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>79</v>
+        <v>126</v>
       </c>
       <c r="C36" s="1" t="b">
         <v>1</v>
@@ -1621,21 +1724,21 @@
         <v>6</v>
       </c>
       <c r="E36">
-        <v>-3</v>
+        <v>0</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>79</v>
+        <v>126</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>80</v>
+        <v>127</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A37" s="4">
+      <c r="A37" s="1">
         <v>36</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="C37" s="1" t="b">
         <v>1</v>
@@ -1647,18 +1750,18 @@
         <v>2</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="G37" s="2" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A38" s="4">
+      <c r="A38" s="1">
         <v>37</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>87</v>
+        <v>118</v>
       </c>
       <c r="C38" s="1" t="b">
         <v>1</v>
@@ -1670,18 +1773,18 @@
         <v>0</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>87</v>
+        <v>118</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A39" s="4">
+      <c r="A39" s="1">
         <v>38</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="C39" s="1" t="b">
         <v>1</v>
@@ -1693,18 +1796,18 @@
         <v>2</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="G39" s="2" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A40" s="4">
+      <c r="A40" s="1">
         <v>39</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="C40" s="1" t="b">
         <v>1</v>
@@ -1716,18 +1819,18 @@
         <v>2</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A41" s="4">
+      <c r="A41" s="1">
         <v>40</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
       <c r="C41" s="1" t="b">
         <v>1</v>
@@ -1739,18 +1842,18 @@
         <v>1</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
       <c r="G41" s="2" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A42" s="4">
+      <c r="A42" s="1">
         <v>41</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="C42" s="1" t="b">
         <v>1</v>
@@ -1762,18 +1865,18 @@
         <v>2</v>
       </c>
       <c r="F42" s="2" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="G42" s="2" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A43" s="4">
+      <c r="A43" s="1">
         <v>42</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="C43" s="1" t="b">
         <v>1</v>
@@ -1785,18 +1888,18 @@
         <v>0</v>
       </c>
       <c r="F43" s="2" t="s">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="G43" s="2" t="s">
-        <v>101</v>
+        <v>92</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A44" s="4">
+      <c r="A44" s="1">
         <v>43</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>99</v>
+        <v>90</v>
       </c>
       <c r="C44" s="1" t="b">
         <v>1</v>
@@ -1808,10 +1911,286 @@
         <v>6</v>
       </c>
       <c r="F44" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="G44" s="2" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A45" s="1">
+        <v>44</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="C45" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="D45" s="2">
+        <v>8</v>
+      </c>
+      <c r="E45">
+        <v>2</v>
+      </c>
+      <c r="F45" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="G45" s="2" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A46" s="1">
+        <v>45</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="C46" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="D46" s="2">
+        <v>10</v>
+      </c>
+      <c r="E46">
+        <v>3</v>
+      </c>
+      <c r="F46" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="G46" s="2" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A47" s="1">
+        <v>46</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="C47" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="D47" s="2">
+        <v>6</v>
+      </c>
+      <c r="E47">
+        <v>1</v>
+      </c>
+      <c r="F47" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="G47" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="G44" s="2" t="s">
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A48" s="1">
+        <v>47</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="C48" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="D48" s="2">
+        <v>6</v>
+      </c>
+      <c r="E48">
+        <v>0</v>
+      </c>
+      <c r="F48" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="G48" s="2" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A49" s="1">
+        <v>48</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="C49" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="D49" s="2">
+        <v>6</v>
+      </c>
+      <c r="E49">
+        <v>2</v>
+      </c>
+      <c r="F49" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="G49" s="2" t="s">
         <v>102</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A50" s="1">
+        <v>49</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="C50" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="D50" s="2">
+        <v>5</v>
+      </c>
+      <c r="E50">
+        <v>0</v>
+      </c>
+      <c r="F50" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="G50" s="2" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A51" s="1">
+        <v>50</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="C51" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="D51" s="2">
+        <v>10</v>
+      </c>
+      <c r="E51">
+        <v>3</v>
+      </c>
+      <c r="F51" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="G51" s="2" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A52" s="1">
+        <v>51</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="C52" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="D52" s="2">
+        <v>10</v>
+      </c>
+      <c r="E52">
+        <v>3</v>
+      </c>
+      <c r="F52" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="G52" s="2" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A53" s="1">
+        <v>52</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="C53" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="D53" s="2">
+        <v>8</v>
+      </c>
+      <c r="E53">
+        <v>1</v>
+      </c>
+      <c r="F53" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="G53" s="2" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A54" s="1">
+        <v>53</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="C54" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="D54" s="2">
+        <v>5</v>
+      </c>
+      <c r="E54">
+        <v>0</v>
+      </c>
+      <c r="F54" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="G54" s="2" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A55" s="1">
+        <v>54</v>
+      </c>
+      <c r="B55" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="C55" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="D55" s="2">
+        <v>4</v>
+      </c>
+      <c r="E55">
+        <v>1</v>
+      </c>
+      <c r="F55" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="G55" s="2" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A56" s="4">
+        <v>55</v>
+      </c>
+      <c r="B56" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="C56" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="D56" s="2">
+        <v>4</v>
+      </c>
+      <c r="E56">
+        <v>0</v>
+      </c>
+      <c r="F56" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="G56" s="2" t="s">
+        <v>125</v>
       </c>
     </row>
   </sheetData>
@@ -1852,7 +2231,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C2">
         <v>-2</v>
@@ -1863,16 +2242,16 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="C3">
         <v>0</v>
       </c>
       <c r="D3" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="E3" t="s">
-        <v>65</v>
+        <v>122</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.4">
@@ -1880,16 +2259,16 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="C4">
         <v>0</v>
       </c>
       <c r="D4" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="E4" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.4">
@@ -1897,16 +2276,16 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>70</v>
+        <v>121</v>
       </c>
       <c r="C5">
         <v>0</v>
       </c>
       <c r="D5" t="s">
-        <v>71</v>
+        <v>121</v>
       </c>
       <c r="E5" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>
@@ -1946,16 +2325,16 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="C2">
         <v>0</v>
       </c>
       <c r="D2" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="E2" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
   </sheetData>

</xml_diff>